<commit_message>
chore: quarterly data update 2026-07-01
</commit_message>
<xml_diff>
--- a/data/lamadeleine_locations.xlsx
+++ b/data/lamadeleine_locations.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H88"/>
+  <dimension ref="A1:H87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1491,69 +1491,69 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>East Cobb</t>
+          <t>DFW</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>30062</t>
+          <t>75261</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>4101 Roswell Road</t>
+          <t>3200 E. Airfield Drive</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Suite 812</t>
+          <t>Terminal A Gate A25</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>4101 Roswell Road, Suite 812, Marietta, GA, 30062</t>
+          <t>3200 E. Airfield Drive, Terminal A Gate A25, Dallas, TX, 75261</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Marietta</t>
+          <t>Dallas</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>GA</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>marietta-east-cobb</t>
+          <t>dfw</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>DFW</t>
+          <t>Dallas Love Field</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>75261</t>
+          <t>75235</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>3200 E. Airfield Drive</t>
+          <t>8008 Cedar Springs Rd.</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Terminal A Gate A25</t>
+          <t>Terminal 2 Gate 6</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>3200 E. Airfield Drive, Terminal A Gate A25, Dallas, TX, 75261</t>
+          <t>8008 Cedar Springs Rd., Terminal 2 Gate 6, Dallas, TX, 75235</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1568,431 +1568,427 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>dfw</t>
+          <t>dallas-love-field</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Dallas Love Field</t>
+          <t>Columbia</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>75235</t>
+          <t>21045</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>8008 Cedar Springs Rd.</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>Terminal 2 Gate 6</t>
-        </is>
-      </c>
+          <t>6211 Columbia Crossing</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>8008 Cedar Springs Rd., Terminal 2 Gate 6, Dallas, TX, 75235</t>
+          <t>6211 Columbia Crossing, Columbia, MD, 21045</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Dallas</t>
+          <t>Columbia</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>MD</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>dallas-love-field</t>
+          <t>columbia</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Columbia</t>
+          <t>Collin Creek</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>21045</t>
+          <t>75075</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>6211 Columbia Crossing</t>
+          <t>520 W. 15th Street</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>6211 Columbia Crossing, Columbia, MD, 21045</t>
+          <t>520 W. 15th Street, Plano, TX, 75075</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Columbia</t>
+          <t>Plano</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>MD</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>columbia</t>
+          <t>plano-collin-creek</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Collin Creek</t>
+          <t>Buford</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>75075</t>
+          <t>30519</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>520 W. 15th Street</t>
+          <t>1795 Mall of Georgia Boulevard</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>520 W. 15th Street, Plano, TX, 75075</t>
+          <t>1795 Mall of Georgia Boulevard, Buford, GA, 30519</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Plano</t>
+          <t>Buford</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>GA</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>plano-collin-creek</t>
+          <t>buford</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Buford</t>
+          <t>Bethesda</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>30519</t>
+          <t>20814</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>1795 Mall of Georgia Boulevard</t>
+          <t>7607 Old Georgetown Road</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>1795 Mall of Georgia Boulevard, Buford, GA, 30519</t>
+          <t>7607 Old Georgetown Road, Bethesda, MD, 20814</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Buford</t>
+          <t>Bethesda</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>GA</t>
+          <t>MD</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>buford</t>
+          <t>baileys-crossroads</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Bethesda</t>
+          <t>Bailey's Crossroads</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>20814</t>
+          <t>22041</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>7607 Old Georgetown Road</t>
+          <t>5861 Crossroads Center Way</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>7607 Old Georgetown Road, Bethesda, MD, 20814</t>
+          <t>5861 Crossroads Center Way, Bailey's Crossroads, VA, 22041</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Bethesda</t>
+          <t>Bailey's Crossroads</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>MD</t>
+          <t>VA</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>baileys-crossroads</t>
+          <t>baileys-crossroads-2</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Bailey's Crossroads</t>
+          <t>Gwinnett</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>22041</t>
+          <t>30096</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>5861 Crossroads Center Way</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr"/>
+          <t>2255 Pleasant Hill Road</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Suite 480</t>
+        </is>
+      </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>5861 Crossroads Center Way, Bailey's Crossroads, VA, 22041</t>
+          <t>2255 Pleasant Hill Road, Suite 480, Duluth, GA, 30096</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Bailey's Crossroads</t>
+          <t>Duluth</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>VA</t>
+          <t>GA</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>baileys-crossroads-2</t>
+          <t>duluth-gwinnett</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Gwinnett</t>
+          <t>Kingsgate</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>30096</t>
+          <t>79424</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2255 Pleasant Hill Road</t>
+          <t>8201 Quaker Avenue</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Suite 480</t>
+          <t>Suite 118</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2255 Pleasant Hill Road, Suite 480, Duluth, GA, 30096</t>
+          <t>8201 Quaker Avenue, Suite 118, Lubbock, TX, 79424</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Duluth</t>
+          <t>Lubbock</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>GA</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>duluth-gwinnett</t>
+          <t>lubbock-kingsgate</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Kingsgate</t>
+          <t>West Little Rock</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>79424</t>
+          <t>72211</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>8201 Quaker Avenue</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>Suite 118</t>
-        </is>
-      </c>
+          <t>12210 W. Markham Drive</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>8201 Quaker Avenue, Suite 118, Lubbock, TX, 79424</t>
+          <t>12210 W. Markham Drive, Little Rock, AR, 72211</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Lubbock</t>
+          <t>Little Rock</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>lubbock-kingsgate</t>
+          <t>little-rock</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>West Little Rock</t>
+          <t>Mandeville</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>72211</t>
+          <t>70471</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>12210 W. Markham Drive</t>
+          <t>3434 Highway 190</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>12210 W. Markham Drive, Little Rock, AR, 72211</t>
+          <t>3434 Highway 190, Mandeville, LA, 70471</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Little Rock</t>
+          <t>Mandeville</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>LA</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>little-rock</t>
+          <t>mandeville</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Mandeville</t>
+          <t>Tanglewood</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>70471</t>
+          <t>77057</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>3434 Highway 190</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr"/>
+          <t>5885 San Felipe Street</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Suite 100</t>
+        </is>
+      </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>3434 Highway 190, Mandeville, LA, 70471</t>
+          <t>5885 San Felipe Street, Suite 100, Houston, TX, 77057</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Mandeville</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>LA</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>mandeville</t>
+          <t>houston-tanglewood</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Tanglewood</t>
+          <t>Tyler</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>77057</t>
+          <t>75701</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>5885 San Felipe Street</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>Suite 100</t>
-        </is>
-      </c>
+          <t>419 WSW Loop 323</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
-          <t>5885 San Felipe Street, Suite 100, Houston, TX, 77057</t>
+          <t>419 WSW Loop 323, Tyler, TX, 75701</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Tyler</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2002,100 +1998,104 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>houston-tanglewood</t>
+          <t>tyler</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Tyler</t>
+          <t>Tulsa Hills</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>75701</t>
+          <t>74107</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>419 WSW Loop 323</t>
+          <t>8115 S. Olympia Avenue West</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
-          <t>419 WSW Loop 323, Tyler, TX, 75701</t>
+          <t>8115 S. Olympia Avenue West, Tulsa, OK, 74107</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Tyler</t>
+          <t>Tulsa</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>tyler</t>
+          <t>tulsa-hills</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Tulsa Hills</t>
+          <t>Town &amp; Country</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>74107</t>
+          <t>77024</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>8115 S. Olympia Avenue West</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr"/>
+          <t>770 W. Sam Houston Parkway N.</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Suite 100</t>
+        </is>
+      </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>8115 S. Olympia Avenue West, Tulsa, OK, 74107</t>
+          <t>770 W. Sam Houston Parkway N., Suite 100, Houston, TX, 77024</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Tulsa</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>tulsa-hills</t>
+          <t>houston-town-country</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Town &amp; Country</t>
+          <t>The Forum</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>77024</t>
+          <t>78154</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>770 W. Sam Houston Parkway N.</t>
+          <t>8134 Agora Parkway</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -2105,12 +2105,12 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>770 W. Sam Houston Parkway N., Suite 100, Houston, TX, 77024</t>
+          <t>8134 Agora Parkway, Suite 100, Live Oak, TX, 78154</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Live Oak</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -2120,39 +2120,35 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>houston-town-country</t>
+          <t>live-oak-the-forum</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>The Forum</t>
+          <t>Sunset Valley</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>78154</t>
+          <t>78745</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>8134 Agora Parkway</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>Suite 100</t>
-        </is>
-      </c>
+          <t>5493 Brodie Lane</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
-          <t>8134 Agora Parkway, Suite 100, Live Oak, TX, 78154</t>
+          <t>5493 Brodie Lane, Austin, TX, 78745</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Live Oak</t>
+          <t>Austin</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2162,35 +2158,39 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>live-oak-the-forum</t>
+          <t>austin-sunset-valley</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Sunset Valley</t>
+          <t>South Arlington</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>78745</t>
+          <t>76015</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>5493 Brodie Lane</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr"/>
+          <t>4201 S. Cooper Street</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Suite 731</t>
+        </is>
+      </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>5493 Brodie Lane, Austin, TX, 78745</t>
+          <t>4201 S. Cooper Street, Suite 731, Arlington, TX, 76015</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Austin</t>
+          <t>Arlington</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -2200,77 +2200,77 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>austin-sunset-valley</t>
+          <t>south-arlington</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>South Arlington</t>
+          <t>Shops at Martial</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>76015</t>
+          <t>70508</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>4201 S. Cooper Street</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>Suite 731</t>
-        </is>
-      </c>
+          <t>2207-I Kaliste Saloom Road</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
-          <t>4201 S. Cooper Street, Suite 731, Arlington, TX, 76015</t>
+          <t>2207-I Kaliste Saloom Road, Lafayette, LA, 70508</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Arlington</t>
+          <t>Lafayette</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>LA</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>south-arlington</t>
+          <t>lafayette-shops-at-martial</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Shops at Martial</t>
+          <t>Severn</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>70508</t>
+          <t>70002</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2207-I Kaliste Saloom Road</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr"/>
+          <t>3300 Severn</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Suite 201</t>
+        </is>
+      </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>2207-I Kaliste Saloom Road, Lafayette, LA, 70508</t>
+          <t>3300 Severn, Suite 201, Metairie, LA, 70002</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Lafayette</t>
+          <t>Metairie</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2280,123 +2280,119 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>lafayette-shops-at-martial</t>
+          <t>metairie-severn</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Severn</t>
+          <t>San Tan Village</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>70002</t>
+          <t>85296</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>3300 Severn</t>
+          <t>2156 E. Williams Field Rd.</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Suite 201</t>
+          <t>Suite 101</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>3300 Severn, Suite 201, Metairie, LA, 70002</t>
+          <t>2156 E. Williams Field Rd., Suite 101, Gilbert, AZ, 85296</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Metairie</t>
+          <t>Gilbert</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>LA</t>
+          <t>AZ</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>metairie-severn</t>
+          <t>gilbert-san-tan-village</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>San Tan Village</t>
+          <t>San Jacinto</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>85296</t>
+          <t>75201</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>2156 E. Williams Field Rd.</t>
+          <t>2100 Ross Avenue</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Suite 101</t>
+          <t>Suite 120</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>2156 E. Williams Field Rd., Suite 101, Gilbert, AZ, 85296</t>
+          <t>2100 Ross Avenue, Suite 120, Dallas, TX, 75201</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Gilbert</t>
+          <t>Dallas</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>AZ</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>gilbert-san-tan-village</t>
+          <t>dallas-san-jacinto</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>San Jacinto</t>
+          <t>Rockwall</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>75201</t>
+          <t>75087</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>2100 Ross Avenue</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>Suite 120</t>
-        </is>
-      </c>
+          <t>987 East I-30</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr">
         <is>
-          <t>2100 Ross Avenue, Suite 120, Dallas, TX, 75201</t>
+          <t>987 East I-30, Rockwall, TX, 75087</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Dallas</t>
+          <t>Rockwall</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -2406,35 +2402,35 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>dallas-san-jacinto</t>
+          <t>rockwall</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Rockwall</t>
+          <t>River Oaks</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>75087</t>
+          <t>77019</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>987 East I-30</t>
+          <t>2047-A West Gray</t>
         </is>
       </c>
       <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr">
         <is>
-          <t>987 East I-30, Rockwall, TX, 75087</t>
+          <t>2047-A West Gray, Houston, TX, 77019</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Rockwall</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -2444,35 +2440,39 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>rockwall</t>
+          <t>houston-river-oaks</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>River Oaks</t>
+          <t>Preston Forest</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>77019</t>
+          <t>75230</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>2047-A West Gray</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr"/>
+          <t>11930 Preston Road</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Suite 100</t>
+        </is>
+      </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>2047-A West Gray, Houston, TX, 77019</t>
+          <t>11930 Preston Road, Suite 100, Dallas, TX, 75230</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Dallas</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -2482,24 +2482,24 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>houston-river-oaks</t>
+          <t>dallas-preston-forest</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Preston Forest</t>
+          <t>Plano</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>75230</t>
+          <t>75093</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>11930 Preston Road</t>
+          <t>5000 W. Park Boulevard</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -2509,12 +2509,12 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>11930 Preston Road, Suite 100, Dallas, TX, 75230</t>
+          <t>5000 W. Park Boulevard, Suite 100, Plano, TX, 75093</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Dallas</t>
+          <t>Plano</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -2524,153 +2524,153 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>dallas-preston-forest</t>
+          <t>plano</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Plano</t>
+          <t>Uptown</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>75093</t>
+          <t>87110</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>5000 W. Park Boulevard</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>Suite 100</t>
-        </is>
-      </c>
+          <t>2110 Louisiana Blvd. NE</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr"/>
       <c r="E53" t="inlineStr">
         <is>
-          <t>5000 W. Park Boulevard, Suite 100, Plano, TX, 75093</t>
+          <t>2110 Louisiana Blvd. NE, Albuquerque, NM, 87110</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Plano</t>
+          <t>Albuquerque</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>NM</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>plano</t>
+          <t>albuquerque-uptown</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Uptown</t>
+          <t>Alexandria</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>87110</t>
+          <t>22314</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>2110 Louisiana Blvd. NE</t>
+          <t>500 King Street</t>
         </is>
       </c>
       <c r="D54" t="inlineStr"/>
       <c r="E54" t="inlineStr">
         <is>
-          <t>2110 Louisiana Blvd. NE, Albuquerque, NM, 87110</t>
+          <t>500 King Street, Alexandria, VA, 22314</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Albuquerque</t>
+          <t>Alexandria</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>NM</t>
+          <t>VA</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>albuquerque-uptown</t>
+          <t>alexandria</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Alexandria</t>
+          <t>Allen</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>22314</t>
+          <t>75013</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>500 King Street</t>
+          <t>810 W. McDermott Drive</t>
         </is>
       </c>
       <c r="D55" t="inlineStr"/>
       <c r="E55" t="inlineStr">
         <is>
-          <t>500 King Street, Alexandria, VA, 22314</t>
+          <t>810 W. McDermott Drive, Allen, TX, 75013</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Alexandria</t>
+          <t>Allen</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>VA</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>alexandria</t>
+          <t>allen</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Allen</t>
+          <t>Arboretum</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>75013</t>
+          <t>78759</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>810 W. McDermott Drive</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr"/>
+          <t>9828 Great Hills Trail</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Suite 650</t>
+        </is>
+      </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>810 W. McDermott Drive, Allen, TX, 75013</t>
+          <t>9828 Great Hills Trail, Suite 650, Austin, TX, 78759</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Allen</t>
+          <t>Austin</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -2680,39 +2680,35 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>allen</t>
+          <t>austin-arboretum</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Arboretum</t>
+          <t>Camp Bowie</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>78759</t>
+          <t>76116</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>9828 Great Hills Trail</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>Suite 650</t>
-        </is>
-      </c>
+          <t>6140 Camp Bowie</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr"/>
       <c r="E57" t="inlineStr">
         <is>
-          <t>9828 Great Hills Trail, Suite 650, Austin, TX, 78759</t>
+          <t>6140 Camp Bowie, Ft. Worth, TX, 76116</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Austin</t>
+          <t>Ft. Worth</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -2722,35 +2718,39 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>austin-arboretum</t>
+          <t>fort-worth-camp-bowie</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Camp Bowie</t>
+          <t>Carillon</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>76116</t>
+          <t>77042</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>6140 Camp Bowie</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr"/>
+          <t>10001 Westheimer Road</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Suite 2123</t>
+        </is>
+      </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>6140 Camp Bowie, Ft. Worth, TX, 76116</t>
+          <t>10001 Westheimer Road, Suite 2123, Houston, TX, 77042</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Ft. Worth</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -2760,115 +2760,111 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>fort-worth-camp-bowie</t>
+          <t>houston-carillon</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Carillon</t>
+          <t>Carrollton</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>77042</t>
+          <t>70118</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>10001 Westheimer Road</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>Suite 2123</t>
-        </is>
-      </c>
+          <t>601 S. Carrollton Avenue</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr"/>
       <c r="E59" t="inlineStr">
         <is>
-          <t>10001 Westheimer Road, Suite 2123, Houston, TX, 77042</t>
+          <t>601 S. Carrollton Avenue, New Orleans, LA, 70118</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>New Orleans</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>LA</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>houston-carillon</t>
+          <t>new-orleans-carrollton</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Carrollton</t>
+          <t>Champions</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>70118</t>
+          <t>77069</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>601 S. Carrollton Avenue</t>
+          <t>5505-A FM 1960</t>
         </is>
       </c>
       <c r="D60" t="inlineStr"/>
       <c r="E60" t="inlineStr">
         <is>
-          <t>601 S. Carrollton Avenue, New Orleans, LA, 70118</t>
+          <t>5505-A FM 1960, Houston, TX, 77069</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>New Orleans</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>LA</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>new-orleans-carrollton</t>
+          <t>houston-champions</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Champions</t>
+          <t>Clearlake</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>77069</t>
+          <t>77598</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>5505-A FM 1960</t>
+          <t>929 West Bay Area Boulevard</t>
         </is>
       </c>
       <c r="D61" t="inlineStr"/>
       <c r="E61" t="inlineStr">
         <is>
-          <t>5505-A FM 1960, Houston, TX, 77069</t>
+          <t>929 West Bay Area Boulevard, Webster, TX, 77598</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Webster</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -2878,35 +2874,35 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>houston-champions</t>
+          <t>webster-clearlake</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Clearlake</t>
+          <t>Coit &amp; Campbell</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>77598</t>
+          <t>75080</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>929 West Bay Area Boulevard</t>
+          <t>1320 W. Campbell</t>
         </is>
       </c>
       <c r="D62" t="inlineStr"/>
       <c r="E62" t="inlineStr">
         <is>
-          <t>929 West Bay Area Boulevard, Webster, TX, 77598</t>
+          <t>1320 W. Campbell, Richardson, TX, 75080</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Webster</t>
+          <t>Richardson</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -2916,35 +2912,39 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>webster-clearlake</t>
+          <t>richardson-coit-campbell</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Coit &amp; Campbell</t>
+          <t>Crossroads</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>75080</t>
+          <t>77065</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>1320 W. Campbell</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr"/>
+          <t>19710 Northwest Freeway (290)</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Suite 100</t>
+        </is>
+      </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>1320 W. Campbell, Richardson, TX, 75080</t>
+          <t>19710 Northwest Freeway (290), Suite 100, Houston, TX, 77065</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Richardson</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -2954,119 +2954,119 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>richardson-coit-campbell</t>
+          <t>houston-crossroads</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Crossroads</t>
+          <t>Downtown Crown</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>77065</t>
+          <t>20878</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>19710 Northwest Freeway (290)</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>Suite 100</t>
-        </is>
-      </c>
+          <t>242 Crown Park Avenue</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr"/>
       <c r="E64" t="inlineStr">
         <is>
-          <t>19710 Northwest Freeway (290), Suite 100, Houston, TX, 77065</t>
+          <t>242 Crown Park Avenue, Gaithersburg, MD, 20878</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Gaithersburg</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>MD</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>houston-crossroads</t>
+          <t>gaithersburg-downtown-crown</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Downtown Crown</t>
+          <t>Flower Mound</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>20878</t>
+          <t>75028</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>242 Crown Park Avenue</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr"/>
+          <t>2500 Cross Timbers Road</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Suite 150</t>
+        </is>
+      </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>242 Crown Park Avenue, Gaithersburg, MD, 20878</t>
+          <t>2500 Cross Timbers Road, Suite 150, Flower Mound, TX, 75028</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Gaithersburg</t>
+          <t>Flower Mound</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>MD</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>gaithersburg-downtown-crown</t>
+          <t>flower-mound</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Flower Mound</t>
+          <t>Frisco</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>75028</t>
+          <t>75034</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>2500 Cross Timbers Road</t>
+          <t>8008 State Hwy 121</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Suite 150</t>
+          <t>Suite 100</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>2500 Cross Timbers Road, Suite 150, Flower Mound, TX, 75028</t>
+          <t>8008 State Hwy 121, Suite 100, Frisco, TX, 75034</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Flower Mound</t>
+          <t>Frisco</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -3076,39 +3076,35 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>flower-mound</t>
+          <t>frisco</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Frisco</t>
+          <t>Grapevine</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>75034</t>
+          <t>76051</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>8008 State Hwy 121</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>Suite 100</t>
-        </is>
-      </c>
+          <t>900 W. State Highway 114</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr"/>
       <c r="E67" t="inlineStr">
         <is>
-          <t>8008 State Hwy 121, Suite 100, Frisco, TX, 75034</t>
+          <t>900 W. State Highway 114, Grapevine, TX, 76051</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Frisco</t>
+          <t>Grapevine</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -3118,35 +3114,39 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>frisco</t>
+          <t>grapevine</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Grapevine</t>
+          <t>Huebner Oaks</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>76051</t>
+          <t>78230</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>900 W. State Highway 114</t>
-        </is>
-      </c>
-      <c r="D68" t="inlineStr"/>
+          <t>11745 Hwy. 10 West</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Suite 101</t>
+        </is>
+      </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>900 W. State Highway 114, Grapevine, TX, 76051</t>
+          <t>11745 Hwy. 10 West, Suite 101, San Antonio, TX, 78230</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Grapevine</t>
+          <t>San Antonio</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -3156,157 +3156,157 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>grapevine</t>
+          <t>san-antonio-huebner-oaks</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Huebner Oaks</t>
+          <t>Jefferson</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>78230</t>
+          <t>70809</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>11745 Hwy. 10 West</t>
-        </is>
-      </c>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>Suite 101</t>
-        </is>
-      </c>
+          <t>7615 Jefferson Highway</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr"/>
       <c r="E69" t="inlineStr">
         <is>
-          <t>11745 Hwy. 10 West, Suite 101, San Antonio, TX, 78230</t>
+          <t>7615 Jefferson Highway, Baton Rouge, LA, 70809</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>San Antonio</t>
+          <t>Baton Rouge</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>LA</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>san-antonio-huebner-oaks</t>
+          <t>baton-rouge-jefferson</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Jefferson</t>
+          <t>Kingstowne</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>70809</t>
+          <t>22315</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>7615 Jefferson Highway</t>
-        </is>
-      </c>
-      <c r="D70" t="inlineStr"/>
+          <t>5876 Kingstowne Center</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Suite 100</t>
+        </is>
+      </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>7615 Jefferson Highway, Baton Rouge, LA, 70809</t>
+          <t>5876 Kingstowne Center, Suite 100, Alexandria, VA, 22315</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>Baton Rouge</t>
+          <t>Alexandria</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>LA</t>
+          <t>VA</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>baton-rouge-jefferson</t>
+          <t>alexandria-kingstowne</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Kingstowne</t>
+          <t>Kingwood</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>22315</t>
+          <t>77345</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>5876 Kingstowne Center</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t>Suite 100</t>
-        </is>
-      </c>
+          <t>4570 Kingwood Drive</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr"/>
       <c r="E71" t="inlineStr">
         <is>
-          <t>5876 Kingstowne Center, Suite 100, Alexandria, VA, 22315</t>
+          <t>4570 Kingwood Drive, Kingwood, TX, 77345</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Alexandria</t>
+          <t>Kingwood</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>VA</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>alexandria-kingstowne</t>
+          <t>kingwood</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Kingwood</t>
+          <t>Lakeline</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>77345</t>
+          <t>78717</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>4570 Kingwood Drive</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr"/>
+          <t>14028 N. US Hwy 183</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Suite 210</t>
+        </is>
+      </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>4570 Kingwood Drive, Kingwood, TX, 77345</t>
+          <t>14028 N. US Hwy 183, Suite 210, Austin, TX, 78717</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Kingwood</t>
+          <t>Austin</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -3316,119 +3316,119 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>kingwood</t>
+          <t>austin-lakeline</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Lakeline</t>
+          <t>Luhrs City Center</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>78717</t>
+          <t>85003</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>14028 N. US Hwy 183</t>
+          <t>45 West Jefferson Street</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Suite 210</t>
+          <t>Suite M</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>14028 N. US Hwy 183, Suite 210, Austin, TX, 78717</t>
+          <t>45 West Jefferson Street, Suite M, Phoenix, AZ, 85003</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Austin</t>
+          <t>Phoenix</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>AZ</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>austin-lakeline</t>
+          <t>phoenix-luhrs-city-center</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Luhrs City Center</t>
+          <t>MacArthur</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>85003</t>
+          <t>75039</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>45 West Jefferson Street</t>
-        </is>
-      </c>
-      <c r="D74" t="inlineStr">
-        <is>
-          <t>Suite M</t>
-        </is>
-      </c>
+          <t>6430 North MacArthur Boulevard</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr"/>
       <c r="E74" t="inlineStr">
         <is>
-          <t>45 West Jefferson Street, Suite M, Phoenix, AZ, 85003</t>
+          <t>6430 North MacArthur Boulevard, Irving, TX, 75039</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Phoenix</t>
+          <t>Irving</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>AZ</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>phoenix-luhrs-city-center</t>
+          <t>irving-macarthur</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>MacArthur</t>
+          <t>Meyerland</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>75039</t>
+          <t>77096</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>6430 North MacArthur Boulevard</t>
-        </is>
-      </c>
-      <c r="D75" t="inlineStr"/>
+          <t>4700 Beechnut</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Suite 620</t>
+        </is>
+      </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>6430 North MacArthur Boulevard, Irving, TX, 75039</t>
+          <t>4700 Beechnut, Suite 620, Houston, TX, 77096</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Irving</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -3438,39 +3438,39 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>irving-macarthur</t>
+          <t>houston-meyerland</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Meyerland</t>
+          <t>Midway</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>77096</t>
+          <t>75220</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>4700 Beechnut</t>
+          <t>4343 W. Northwest Hwy</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Suite 620</t>
+          <t>Suite 365</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>4700 Beechnut, Suite 620, Houston, TX, 77096</t>
+          <t>4343 W. Northwest Hwy, Suite 365, Dallas, TX, 75220</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Dallas</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -3480,34 +3480,30 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>houston-meyerland</t>
+          <t>dallas-midway</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Midway</t>
+          <t>Mockingbird</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>75220</t>
+          <t>75205</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>4343 W. Northwest Hwy</t>
-        </is>
-      </c>
-      <c r="D77" t="inlineStr">
-        <is>
-          <t>Suite 365</t>
-        </is>
-      </c>
+          <t>3072 Mockingbird Lane</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr"/>
       <c r="E77" t="inlineStr">
         <is>
-          <t>4343 W. Northwest Hwy, Suite 365, Dallas, TX, 75220</t>
+          <t>3072 Mockingbird Lane, Dallas, TX, 75205</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -3522,35 +3518,39 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>dallas-midway</t>
+          <t>dallas-mockingbird</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Mockingbird</t>
+          <t>Mueller</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>75205</t>
+          <t>78723</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>3072 Mockingbird Lane</t>
-        </is>
-      </c>
-      <c r="D78" t="inlineStr"/>
+          <t>1201  Barbara Jordan Boulevard</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Bldg 11, Ste 100</t>
+        </is>
+      </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>3072 Mockingbird Lane, Dallas, TX, 75205</t>
+          <t>1201  Barbara Jordan Boulevard, Bldg 11, Ste 100, Austin, TX, 78723</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Dallas</t>
+          <t>Austin</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -3560,39 +3560,35 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>dallas-mockingbird</t>
+          <t>austin-mueller</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Mueller</t>
+          <t>North Arlington</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>78723</t>
+          <t>76011</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>1201  Barbara Jordan Boulevard</t>
-        </is>
-      </c>
-      <c r="D79" t="inlineStr">
-        <is>
-          <t>Bldg 11, Ste 100</t>
-        </is>
-      </c>
+          <t>2101 N. Collins</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr"/>
       <c r="E79" t="inlineStr">
         <is>
-          <t>1201  Barbara Jordan Boulevard, Bldg 11, Ste 100, Austin, TX, 78723</t>
+          <t>2101 N. Collins, Arlington, TX, 76011</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Austin</t>
+          <t>Arlington</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -3602,35 +3598,35 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>austin-mueller</t>
+          <t>north-arlington</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>North Arlington</t>
+          <t>Northwoods</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>76011</t>
+          <t>78232</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>2101 N. Collins</t>
+          <t>18030 US Hwy 281 N</t>
         </is>
       </c>
       <c r="D80" t="inlineStr"/>
       <c r="E80" t="inlineStr">
         <is>
-          <t>2101 N. Collins, Arlington, TX, 76011</t>
+          <t>18030 US Hwy 281 N, San Antonio, TX, 78232</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>Arlington</t>
+          <t>San Antonio</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
@@ -3640,35 +3636,35 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>north-arlington</t>
+          <t>san-antonio-northwoods</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Northwoods</t>
+          <t>Overton Park</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>78232</t>
+          <t>76109</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>18030 US Hwy 281 N</t>
+          <t>4626 SW Loop 820</t>
         </is>
       </c>
       <c r="D81" t="inlineStr"/>
       <c r="E81" t="inlineStr">
         <is>
-          <t>18030 US Hwy 281 N, San Antonio, TX, 78232</t>
+          <t>4626 SW Loop 820, Ft. Worth, TX, 76109</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>San Antonio</t>
+          <t>Ft. Worth</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -3678,35 +3674,39 @@
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>san-antonio-northwoods</t>
+          <t>fort-worth-overton-park</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Overton Park</t>
+          <t>Park North</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>76109</t>
+          <t>78216</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>4626 SW Loop 820</t>
-        </is>
-      </c>
-      <c r="D82" t="inlineStr"/>
+          <t>722 NW Loop 410</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Suite 201</t>
+        </is>
+      </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>4626 SW Loop 820, Ft. Worth, TX, 76109</t>
+          <t>722 NW Loop 410, Suite 201, San Antonio, TX, 78216</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Ft. Worth</t>
+          <t>San Antonio</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
@@ -3716,39 +3716,39 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>fort-worth-overton-park</t>
+          <t>san-antonio-park-north</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Park North</t>
+          <t>Parkway Village</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>78216</t>
+          <t>77077</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>722 NW Loop 410</t>
+          <t>1560 Eldridge Parkway</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Suite 201</t>
+          <t>Suite 190</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>722 NW Loop 410, Suite 201, San Antonio, TX, 78216</t>
+          <t>1560 Eldridge Parkway, Suite 190, Houston, TX, 77077</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>San Antonio</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
@@ -3758,39 +3758,39 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>san-antonio-park-north</t>
+          <t>houston-parkway-village</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Parkway Village</t>
+          <t>Pearland</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>77077</t>
+          <t>77584</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>1560 Eldridge Parkway</t>
+          <t>11200 Broadway Street</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Suite 190</t>
+          <t>Suite 1600</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>1560 Eldridge Parkway, Suite 190, Houston, TX, 77077</t>
+          <t>11200 Broadway Street, Suite 1600, Pearland, TX, 77584</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Pearland</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
@@ -3800,165 +3800,123 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>houston-parkway-village</t>
+          <t>pearland</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Pearland</t>
+          <t>Perkins Rowe</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>77584</t>
+          <t>70810</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>11200 Broadway Street</t>
+          <t>7707 Bluebonnet Boulevard</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Suite 1600</t>
+          <t>Suite 190</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>11200 Broadway Street, Suite 1600, Pearland, TX, 77584</t>
+          <t>7707 Bluebonnet Boulevard, Suite 190, Baton Rouge, LA, 70810</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>Pearland</t>
+          <t>Baton Rouge</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>LA</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>pearland</t>
+          <t>baton-rouge-perkins-rowe</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Perkins Rowe</t>
+          <t>West Grand</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>70810</t>
+          <t>77449</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>7707 Bluebonnet Boulevard</t>
-        </is>
-      </c>
-      <c r="D86" t="inlineStr">
-        <is>
-          <t>Suite 190</t>
-        </is>
-      </c>
+          <t>23322 Mercantile Parkway</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr"/>
       <c r="E86" t="inlineStr">
         <is>
-          <t>7707 Bluebonnet Boulevard, Suite 190, Baton Rouge, LA, 70810</t>
+          <t>23322 Mercantile Parkway, Katy, TX, 77449</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>Baton Rouge</t>
+          <t>Katy</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>LA</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>baton-rouge-perkins-rowe</t>
+          <t>katy-west-grand</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>West Grand</t>
+          <t>Norman</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>77449</t>
+          <t>73069</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>23322 Mercantile Parkway</t>
+          <t>1954 24th Avenue NW</t>
         </is>
       </c>
       <c r="D87" t="inlineStr"/>
       <c r="E87" t="inlineStr">
         <is>
-          <t>23322 Mercantile Parkway, Katy, TX, 77449</t>
+          <t>1954 24th Avenue NW, Norman, OK, 73069</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>Katy</t>
+          <t>Norman</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
-        <is>
-          <t>katy-west-grand</t>
-        </is>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" t="inlineStr">
-        <is>
-          <t>Norman</t>
-        </is>
-      </c>
-      <c r="B88" t="inlineStr">
-        <is>
-          <t>73069</t>
-        </is>
-      </c>
-      <c r="C88" t="inlineStr">
-        <is>
-          <t>1954 24th Avenue NW</t>
-        </is>
-      </c>
-      <c r="D88" t="inlineStr"/>
-      <c r="E88" t="inlineStr">
-        <is>
-          <t>1954 24th Avenue NW, Norman, OK, 73069</t>
-        </is>
-      </c>
-      <c r="F88" t="inlineStr">
-        <is>
-          <t>Norman</t>
-        </is>
-      </c>
-      <c r="G88" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="H88" t="inlineStr">
         <is>
           <t>university-town-center-norman</t>
         </is>

</xml_diff>